<commit_message>
Clean up test notebook, refactor delete_many() to discard_many()
</commit_message>
<xml_diff>
--- a/src/pyetm/templates/input_template.xlsx
+++ b/src/pyetm/templates/input_template.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EFA905D-A7CD-F645-839B-639D04F99116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="4" xr2:uid="{AF0205CE-FE76-0D48-9891-27D9A9214571}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{AF0205CE-FE76-0D48-9891-27D9A9214571}"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="8" r:id="rId1"/>

</xml_diff>

<commit_message>
Collections management, discard and deletion for sessions/scenarios
</commit_message>
<xml_diff>
--- a/src/pyetm/templates/input_template.xlsx
+++ b/src/pyetm/templates/input_template.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EFA905D-A7CD-F645-839B-639D04F99116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="4" xr2:uid="{AF0205CE-FE76-0D48-9891-27D9A9214571}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{AF0205CE-FE76-0D48-9891-27D9A9214571}"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="8" r:id="rId1"/>

</xml_diff>